<commit_message>
rewatched 150 for icr4 yugin
</commit_message>
<xml_diff>
--- a/data/comments/comments_reliy_coded.xlsx
+++ b/data/comments/comments_reliy_coded.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joellattmann/Documents/GitHub/like_dislike/data/comments/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yuginkha/Documents/Mediapsychology/like_dislike/data/comments/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9D2E288-CB0A-7646-AA1E-8497DCA85B78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-3880" yWindow="-21000" windowWidth="38400" windowHeight="21000" xr2:uid="{C1BB1A16-32F0-7443-88B2-C6116B7B62A9}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{C1BB1A16-32F0-7443-88B2-C6116B7B62A9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1657,7 +1657,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1677,7 +1677,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>

</xml_diff>